<commit_message>
Updated description, outcome message and output variables.
</commit_message>
<xml_diff>
--- a/rules/CORE-000842/negative/01/data/unit-test-coreid-CG0213-negative 1.xlsx
+++ b/rules/CORE-000842/negative/01/data/unit-test-coreid-CG0213-negative 1.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -73,20 +73,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -106,22 +94,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -157,7 +129,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -167,9 +139,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +481,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
       <c r="B2" s="4" t="str">
@@ -539,18 +508,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Subject Visits</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>tv.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Trial Visits</v>
       </c>
     </row>
@@ -563,7 +532,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -586,45 +555,45 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>13</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>SVUPDES</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>13</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <v>101</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="str">
         <v>sv.xpt</v>
@@ -633,35 +602,75 @@
         <v>Record</v>
       </c>
       <c r="D4" s="2">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>VISIT</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>EARLY DISCONTINUATION</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>sv.xpt</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="4">
         <v>14</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>SVUPDES</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2">
+    <row r="6">
+      <c r="A6" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D6" s="4">
         <v>14</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F6" s="4">
         <v>201</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>2</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>sv.xpt</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="2">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>VISIT</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>EARLY DISCONTINUATION RETRIEVAL</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -712,7 +721,7 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
       <c r="C2" s="6" t="str">
@@ -861,40 +870,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="8" t="str">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C6" s="8" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="8" t="str">
+      <c r="E6" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="F6" s="8" t="str">
+      <c r="F6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G6" s="8" t="str">
+      <c r="G6" s="4" t="str">
         <v>-3</v>
       </c>
-      <c r="H6" s="8" t="str">
+      <c r="H6" s="4" t="str">
         <v>2012-11-28</v>
       </c>
-      <c r="I6" s="8" t="str">
+      <c r="I6" s="4" t="str">
         <v>2012-11-28</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="4">
         <v>-2</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="4">
         <v>-2</v>
       </c>
-      <c r="L6" s="8" t="str">
+      <c r="L6" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -937,40 +946,40 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="8" t="str">
+      <c r="A8" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C8" s="8" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="4">
         <v>4</v>
       </c>
-      <c r="E8" s="8" t="str">
+      <c r="E8" s="4" t="str">
         <v>WEEK 2</v>
       </c>
-      <c r="F8" s="8" t="str">
+      <c r="F8" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G8" s="8" t="str">
+      <c r="G8" s="4" t="str">
         <v>15</v>
       </c>
-      <c r="H8" s="8" t="str">
+      <c r="H8" s="4" t="str">
         <v>2012-12-13</v>
       </c>
-      <c r="I8" s="8" t="str">
+      <c r="I8" s="4" t="str">
         <v>2012-12-13</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="4">
         <v>14</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8" s="4">
         <v>14</v>
       </c>
-      <c r="L8" s="8" t="str">
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -1014,40 +1023,40 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="8" t="str">
+      <c r="A10" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B10" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C10" s="8" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="4">
         <v>5.01</v>
       </c>
-      <c r="E10" s="8" t="str">
+      <c r="E10" s="4" t="str">
         <v>WEEK 4: UNSCHEDULED 01</v>
       </c>
-      <c r="F10" s="8" t="str">
+      <c r="F10" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H10" s="8" t="str">
+      <c r="G10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H10" s="4" t="str">
         <v>2012-12-28</v>
       </c>
-      <c r="I10" s="8" t="str">
+      <c r="I10" s="4" t="str">
         <v>2012-12-28</v>
       </c>
-      <c r="J10" s="8">
+      <c r="J10" s="4">
         <v>29</v>
       </c>
-      <c r="K10" s="8">
+      <c r="K10" s="4">
         <v>29</v>
       </c>
-      <c r="L10" s="8" t="str">
+      <c r="L10" s="4" t="str">
         <v>UNSCHEDULED LABS</v>
       </c>
     </row>
@@ -1090,40 +1099,40 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B12" s="8" t="str">
+      <c r="A12" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B12" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C12" s="8" t="str">
+      <c r="C12" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="4">
         <v>8</v>
       </c>
-      <c r="E12" s="8" t="str">
+      <c r="E12" s="4" t="str">
         <v>WEEK 8</v>
       </c>
-      <c r="F12" s="8" t="str">
+      <c r="F12" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G12" s="8" t="str">
+      <c r="G12" s="4" t="str">
         <v>57</v>
       </c>
-      <c r="H12" s="8" t="str">
+      <c r="H12" s="4" t="str">
         <v>2013-01-23</v>
       </c>
-      <c r="I12" s="8" t="str">
+      <c r="I12" s="4" t="str">
         <v>2013-01-23</v>
       </c>
-      <c r="J12" s="8">
+      <c r="J12" s="4">
         <v>55</v>
       </c>
-      <c r="K12" s="8">
+      <c r="K12" s="4">
         <v>55</v>
       </c>
-      <c r="L12" s="8" t="str">
+      <c r="L12" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -1137,10 +1146,10 @@
       <c r="C13" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="7">
         <v>101</v>
       </c>
-      <c r="E13" s="4" t="str">
+      <c r="E13" s="7" t="str">
         <v>EARLY DISCONTINUATION</v>
       </c>
       <c r="F13" s="4" t="str">
@@ -1161,45 +1170,45 @@
       <c r="K13" s="4">
         <v>77</v>
       </c>
-      <c r="L13" s="9" t="str">
+      <c r="L13" s="7" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B14" s="8" t="str">
+      <c r="A14" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B14" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C14" s="8" t="str">
+      <c r="C14" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="8">
         <v>201</v>
       </c>
-      <c r="E14" s="8" t="str">
+      <c r="E14" s="7" t="str">
         <v>EARLY DISCONTINUATION RETRIEVAL</v>
       </c>
-      <c r="F14" s="8" t="str">
+      <c r="F14" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G14" s="8" t="str">
-        <v/>
-      </c>
-      <c r="H14" s="8" t="str">
+      <c r="G14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H14" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="I14" s="8" t="str">
+      <c r="I14" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="J14" s="8">
+      <c r="J14" s="4">
         <v>172</v>
       </c>
-      <c r="K14" s="8">
+      <c r="K14" s="4">
         <v>172</v>
       </c>
-      <c r="L14" s="11" t="str">
+      <c r="L14" s="8" t="str">
         <v/>
       </c>
     </row>
@@ -1330,25 +1339,25 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="8" t="str">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="4">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="str">
+      <c r="D6" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="E6" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F6" s="8" t="str">
+      <c r="E6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="4" t="str">
         <v>Day Before Initial Study Treatment</v>
       </c>
-      <c r="G6" s="8" t="str">
+      <c r="G6" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -1376,25 +1385,25 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="8" t="str">
+      <c r="A8" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="4">
         <v>4</v>
       </c>
-      <c r="D8" s="8" t="str">
+      <c r="D8" s="4" t="str">
         <v>WEEK 2</v>
       </c>
-      <c r="E8" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F8" s="8" t="str">
+      <c r="E8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="4" t="str">
         <v>2 Weeks After Start of Study Treatment</v>
       </c>
-      <c r="G8" s="8" t="str">
+      <c r="G8" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -1422,25 +1431,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="8" t="str">
+      <c r="A10" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B10" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="4">
         <v>7</v>
       </c>
-      <c r="D10" s="8" t="str">
+      <c r="D10" s="4" t="str">
         <v>WEEK 6</v>
       </c>
-      <c r="E10" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F10" s="8" t="str">
+      <c r="E10" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F10" s="4" t="str">
         <v>6 Weeks After Start of Study Treatment</v>
       </c>
-      <c r="G10" s="8" t="str">
+      <c r="G10" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -1468,25 +1477,25 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B12" s="8" t="str">
+      <c r="A12" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B12" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="4">
         <v>9</v>
       </c>
-      <c r="D12" s="8" t="str">
+      <c r="D12" s="4" t="str">
         <v>WEEK 12</v>
       </c>
-      <c r="E12" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F12" s="8" t="str">
+      <c r="E12" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F12" s="4" t="str">
         <v>12 Weeks After Start of Study Treatment</v>
       </c>
-      <c r="G12" s="8" t="str">
+      <c r="G12" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -1514,25 +1523,25 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B14" s="8" t="str">
+      <c r="A14" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B14" s="4" t="str">
         <v>TV</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="4">
         <v>11</v>
       </c>
-      <c r="D14" s="8" t="str">
+      <c r="D14" s="4" t="str">
         <v>WEEK 20</v>
       </c>
-      <c r="E14" s="8" t="str">
-        <v/>
-      </c>
-      <c r="F14" s="8" t="str">
+      <c r="E14" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F14" s="4" t="str">
         <v>20 Weeks After Start of Study Treatment</v>
       </c>
-      <c r="G14" s="8" t="str">
+      <c r="G14" s="4" t="str">
         <v/>
       </c>
     </row>

</xml_diff>